<commit_message>
feat(keel): migrate debt+balance from Dune to Envio HyperSync
Keel onto the HyperSync backend (sources: debt+balance). Agent-rate-only, so
debt is a no-op; balance reconstructs the subproxy USDS/sUSDS agent-rate base
from raw Transfer logs via the reorg-safe store. Prices/SSR/DR unchanged.

Parity: all 6 months (2026-01..06) regenerate byte-identical summary.md vs
Dune (agent_rate + sky_revenue unchanged); .xlsx differ only in the
regeneration timestamp. Validated with the submodule at its recorded DR commit.

Co-Authored-By: Claude Opus 4.8 (1M context) <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/settlements/keel/2026-01/keel_settlement_january_2026.xlsx
+++ b/settlements/keel/2026-01/keel_settlement_january_2026.xlsx
@@ -1,17 +1,17 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <workbookProtection/>
   <bookViews>
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Summary" sheetId="1" state="visible" r:id="rId1"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Venues" sheetId="2" state="visible" r:id="rId2"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Sky Revenue" sheetId="3" state="visible" r:id="rId3"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Sky Direct" sheetId="4" state="visible" r:id="rId4"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Debt" sheetId="5" state="visible" r:id="rId5"/>
+    <sheet name="Summary" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet name="Venues" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet name="Sky Revenue" sheetId="3" state="visible" r:id="rId3"/>
+    <sheet name="Sky Direct" sheetId="4" state="visible" r:id="rId4"/>
+    <sheet name="Debt" sheetId="5" state="visible" r:id="rId5"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -624,7 +624,7 @@
       </c>
       <c r="B21" t="inlineStr">
         <is>
-          <t>2026-07-07T14:51:52+00:00</t>
+          <t>2026-07-14T09:33:53+00:00</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
feat(hypersync): Dune→HyperSync debt/balance sources with reorg-safe store; obex + tier-2 pilots (#154)
Co-authored-by: Claude Opus 4.8 (1M context) <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/settlements/keel/2026-01/keel_settlement_january_2026.xlsx
+++ b/settlements/keel/2026-01/keel_settlement_january_2026.xlsx
@@ -1,17 +1,17 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <workbookProtection/>
   <bookViews>
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Summary" sheetId="1" state="visible" r:id="rId1"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Venues" sheetId="2" state="visible" r:id="rId2"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Sky Revenue" sheetId="3" state="visible" r:id="rId3"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Sky Direct" sheetId="4" state="visible" r:id="rId4"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Debt" sheetId="5" state="visible" r:id="rId5"/>
+    <sheet name="Summary" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet name="Venues" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet name="Sky Revenue" sheetId="3" state="visible" r:id="rId3"/>
+    <sheet name="Sky Direct" sheetId="4" state="visible" r:id="rId4"/>
+    <sheet name="Debt" sheetId="5" state="visible" r:id="rId5"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -624,7 +624,7 @@
       </c>
       <c r="B21" t="inlineStr">
         <is>
-          <t>2026-07-07T14:51:52+00:00</t>
+          <t>2026-07-14T09:33:53+00:00</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
feat(dr): HyperSync DR workbook + ref-code attribution in config (submodule 962f9f6) (#160)
Co-authored-by: Claude Opus 5 (1M context) <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/settlements/keel/2026-01/keel_settlement_january_2026.xlsx
+++ b/settlements/keel/2026-01/keel_settlement_january_2026.xlsx
@@ -507,13 +507,13 @@
         </is>
       </c>
       <c r="B6" s="3" t="n">
-        <v>28435.59</v>
+        <v>28500.23</v>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr"/>
       <c r="B7" s="4" t="n">
-        <v>28435.59</v>
+        <v>28500.23</v>
       </c>
     </row>
     <row r="9">
@@ -624,7 +624,7 @@
       </c>
       <c r="B21" t="inlineStr">
         <is>
-          <t>2026-07-14T09:33:53+00:00</t>
+          <t>2026-07-15T11:04:30+00:00</t>
         </is>
       </c>
     </row>

</xml_diff>